<commit_message>
Support the business sample upload file layout
- Upload columns are now found by their heading, so both the FS
  template order and the Sample_data_ABAP.xlsx order (packing list A,
  invoice B, items C-M) are read correctly
- Package values repeated on every row of a package are counted once,
  like merged cells; 'Fetch from ...' placeholders are treated as empty
- New unit tests for the sample layout, placeholders and repeated
  package values; sample file and expected results added to test_data

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0112PqhqihbYdjNWGe6hooZE
</commit_message>
<xml_diff>
--- a/Packing_List_Development/templates/ZSD_EPACK_Upload_Template_v2.xlsx
+++ b/Packing_List_Development/templates/ZSD_EPACK_Upload_Template_v2.xlsx
@@ -8188,7 +8188,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A25"/>
+  <dimension ref="A1:A27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="160" customWidth="1" min="1" max="1"/>
@@ -8201,13 +8201,11 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr"/>
-    </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>1. Only the FIRST sheet ('Format') is read. Keep the heading row (row 1) and the column order A-AL.</t>
+          <t>1. Only the FIRST sheet is read. Row 1 must contain the column headings - columns are found by heading, so their order may differ (e.g. Packing list no in A and invoice in B).</t>
         </is>
       </c>
     </row>
@@ -8284,78 +8282,90 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>8. Quantity should equal STD x Articles - a difference is reported as a warning.</t>
+          <t xml:space="preserve">   Instead of merging, the package values (Article No., Articles, Gross/Net Wt.) may also be repeated on every row of the package - same Article No. + same values = one package.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>9. Column AL Package Type (NEW, optional): Loose Pipes / Boxes / Bundles ... entered on the first line of each run; carried forward.</t>
+          <t>8. Quantity should equal STD x Articles - a difference is reported as a warning.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>10. Multi-line cells (Alt+Enter) are printed line by line: notify parties, Container No, No. of Packages, Description of goods, Declaration.</t>
+          <t>9. Column AL Package Type (NEW, optional): Loose Pipes / Boxes / Bundles ... entered on the first line of each run; carried forward.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>11. Notify parties must be filled from 1 upwards. If any notify party is filled, the format 'with notify party' is printed.</t>
+          <t>10. Multi-line cells (Alt+Enter) are printed line by line: notify parties, Container No, No. of Packages, Description of goods, Declaration.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>12. Product Description (G) and H.S Code (K) may be left empty - they are then taken from the material master of the Part No.</t>
+          <t>11. Notify parties must be filled from 1 upwards. If any notify party is filled, the format 'with notify party' is printed.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>13. Column O (Exporter Ref) is not used - the IEC is read from the company address in SAP (FS logic sheet).</t>
+          <t>12a. A cell reading 'Fetch from logic' / 'Fetch from material master' counts as empty - the value is then taken from SAP.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>14. Description of goods (AG) may be left empty - it is then built from the HSN codes of the billed materials (FS logic sheet).</t>
+          <t>12. Product Description (G) and H.S Code (K) may be left empty - they are then taken from the material master of the Part No.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>15. Dates: DD.MM.YYYY or an Excel date. Numbers: plain Excel numbers; weights are rounded to 3 decimals.</t>
+          <t>13. Column O (Exporter Ref) is not used - the IEC is read from the company address in SAP (FS logic sheet).</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>16. Use 'Validate only' first. After a successful output the data is saved to the Z tables and a log row is written per packing list;</t>
+          <t>14. Description of goods (AG) may be left empty - it is then built from the HSN codes of the billed materials (FS logic sheet).</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t xml:space="preserve">    a packing list uploaded again replaces the saved one and gets the next revision number.</t>
+          <t>15. Dates: DD.MM.YYYY or an Excel date. Numbers: plain Excel numbers; weights are rounded to 3 decimals.</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" t="inlineStr"/>
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>16. Use 'Validate only' first. After a successful output the data is saved to the Z tables and a log row is written per packing list;</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    a packing list uploaded again replaces the saved one and gets the next revision number.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26"/>
+    <row r="27">
+      <c r="A27" t="inlineStr">
         <is>
           <t>See sheet 'Example_90000081' for a filled example (data of PackingList_90000081 Nabil Yemen_BySea - Rev.1.pdf).</t>
         </is>

</xml_diff>